<commit_message>
markdownlint GCP_DATA_ENGINEER_STUDY/WEEK_01_GCS/DAY_00_GCP_FUNDAMENTALS.md markdownlint GCP_DATA_ENGINEER_STUDY/WEEK_01_GCS/DAY_01_LEARNING_AND_LAB.md markdownlint GCP_DATA_ENGINEER_STUDY/WEEK_01_GCS/DAY_01_REVISION_SHEET.md markdownlint GCP_DATA_ENGINEER_STUDY/WEEK_01_GCS/DAY_02_COMPUTE_ENGINE_VM.md
</commit_message>
<xml_diff>
--- a/TAP n NRT directories.xlsx
+++ b/TAP n NRT directories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myoffice.accenture.com/personal/v_brabhaharan_accenture_com/Documents/Documents/VMO2/TAP/Script_Opus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{75BF60A8-BB22-4744-A2CE-ACD735186B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03656DF8-AD99-4364-AC52-876415F14205}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{75BF60A8-BB22-4744-A2CE-ACD735186B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50C1C518-784E-45B2-9146-3922206ECF0A}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4800" yWindow="3110" windowWidth="14400" windowHeight="8170" xr2:uid="{0E8EA9B8-1E59-4C3E-9E23-98E6D03B5A03}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0E8EA9B8-1E59-4C3E-9E23-98E6D03B5A03}"/>
   </bookViews>
   <sheets>
     <sheet name="TAP" sheetId="1" r:id="rId1"/>
@@ -8165,7 +8165,7 @@
   <dimension ref="A1:F627"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.81640625" customWidth="1"/>
     <col min="2" max="3" width="19.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="40.453125" customWidth="1"/>

</xml_diff>